<commit_message>
[200~add usart updata flash
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F403ARGT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F403ARGT7_WorkBench_analysis.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="65">
   <si>
     <t>AT32F403ARGT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-8f1da8.o</t>
+    <t>lto-llvm-d97ef7.o</t>
   </si>
   <si>
     <t>startup_at32f403a_407.o</t>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>_chval.o</t>
+  </si>
+  <si>
+    <t>memcmp.o</t>
   </si>
   <si>
     <t>atoi.o</t>
@@ -296,11 +299,11 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>ram_percent!$A$3:$A$56</c:f>
+              <c:f>ram_percent!$A$3:$A$57</c:f>
               <c:strCache>
-                <c:ptCount val="54"/>
+                <c:ptCount val="55"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-8f1da8.o</c:v>
+                  <c:v>lto-llvm-d97ef7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f403a_407.o</c:v>
@@ -317,7 +320,7 @@
                 <c:pt idx="5">
                   <c:v>errno.o</c:v>
                 </c:pt>
-                <c:pt idx="53">
+                <c:pt idx="54">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -325,29 +328,29 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>ram_percent!$B$3:$B$56</c:f>
+              <c:f>ram_percent!$B$3:$B$57</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="54"/>
+                <c:ptCount val="55"/>
                 <c:pt idx="0">
-                  <c:v>97.79456329345703</c:v>
+                  <c:v>97.96974182128906</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.154927492141724</c:v>
+                  <c:v>1.983765721321106</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0252530574798584</c:v>
+                  <c:v>0.02324725314974785</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.008417685516178608</c:v>
+                  <c:v>0.00774908484891057</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.008417685516178608</c:v>
+                  <c:v>0.00774908484891057</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.008417685516178608</c:v>
-                </c:pt>
-                <c:pt idx="53">
+                  <c:v>0.00774908484891057</c:v>
+                </c:pt>
+                <c:pt idx="54">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -415,11 +418,11 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>flash_percent!$A$3:$A$56</c:f>
+              <c:f>flash_percent!$A$3:$A$57</c:f>
               <c:strCache>
-                <c:ptCount val="54"/>
+                <c:ptCount val="55"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-8f1da8.o</c:v>
+                  <c:v>lto-llvm-d97ef7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mc_w.l</c:v>
@@ -542,42 +545,45 @@
                   <c:v>_chval.o</c:v>
                 </c:pt>
                 <c:pt idx="41">
+                  <c:v>memcmp.o</c:v>
+                </c:pt>
+                <c:pt idx="42">
                   <c:v>atoi.o</c:v>
                 </c:pt>
-                <c:pt idx="42">
+                <c:pt idx="43">
                   <c:v>dfltul.o</c:v>
                 </c:pt>
-                <c:pt idx="43">
+                <c:pt idx="44">
                   <c:v>strncpy.o</c:v>
                 </c:pt>
-                <c:pt idx="44">
+                <c:pt idx="45">
                   <c:v>strchr.o</c:v>
                 </c:pt>
-                <c:pt idx="45">
+                <c:pt idx="46">
                   <c:v>isspace_o.o</c:v>
                 </c:pt>
-                <c:pt idx="46">
+                <c:pt idx="47">
                   <c:v>strlen.o</c:v>
                 </c:pt>
-                <c:pt idx="47">
+                <c:pt idx="48">
                   <c:v>errno.o</c:v>
                 </c:pt>
-                <c:pt idx="48">
+                <c:pt idx="49">
                   <c:v>entry9a.o</c:v>
                 </c:pt>
-                <c:pt idx="49">
+                <c:pt idx="50">
                   <c:v>entry2.o</c:v>
                 </c:pt>
-                <c:pt idx="50">
+                <c:pt idx="51">
                   <c:v>stdout.o</c:v>
                 </c:pt>
-                <c:pt idx="51">
+                <c:pt idx="52">
                   <c:v>entry8a.o</c:v>
                 </c:pt>
-                <c:pt idx="52">
+                <c:pt idx="53">
                   <c:v>entry5.o</c:v>
                 </c:pt>
-                <c:pt idx="53">
+                <c:pt idx="54">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -585,170 +591,173 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>flash_percent!$B$3:$B$56</c:f>
+              <c:f>flash_percent!$B$3:$B$57</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="54"/>
+                <c:ptCount val="55"/>
                 <c:pt idx="0">
-                  <c:v>73.85256958007813</c:v>
+                  <c:v>74.96259307861328</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.59873294830322</c:v>
+                  <c:v>10.15662288665772</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.889259576797485</c:v>
+                  <c:v>3.711838960647583</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.094729900360107</c:v>
+                  <c:v>1.999172329902649</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.464309573173523</c:v>
+                  <c:v>1.397510528564453</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.354236125946045</c:v>
+                  <c:v>1.292458534240723</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.7071381211280823</c:v>
+                  <c:v>0.6748798489570618</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.5703802704811096</c:v>
+                  <c:v>0.5443606376647949</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.5570380091667175</c:v>
+                  <c:v>0.5316270589828491</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.5537024736404419</c:v>
+                  <c:v>0.5284436345100403</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.3802534937858582</c:v>
+                  <c:v>0.3629070818424225</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.3735823929309845</c:v>
+                  <c:v>0.3565402925014496</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.3702468276023865</c:v>
+                  <c:v>0.3533568978309631</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.310206800699234</c:v>
+                  <c:v>0.2960557639598846</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.2635090053081513</c:v>
+                  <c:v>0.2514882385730743</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.235156774520874</c:v>
+                  <c:v>0.2244293689727783</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.1867911964654923</c:v>
+                  <c:v>0.1782701462507248</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.1834556311368942</c:v>
+                  <c:v>0.1750867515802383</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.1634422987699509</c:v>
+                  <c:v>0.1559863686561585</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.1634422987699509</c:v>
+                  <c:v>0.1559863686561585</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.1200800538063049</c:v>
+                  <c:v>0.1146022379398346</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.1067378222942352</c:v>
+                  <c:v>0.1018686518073082</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.09339559823274612</c:v>
+                  <c:v>0.0891350731253624</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.09339559823274612</c:v>
+                  <c:v>0.0891350731253624</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.08005336672067642</c:v>
+                  <c:v>0.076401486992836</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.08005336672067642</c:v>
+                  <c:v>0.076401486992836</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.08005336672067642</c:v>
+                  <c:v>0.076401486992836</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.07338225841522217</c:v>
+                  <c:v>0.0700346976518631</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.06671114265918732</c:v>
+                  <c:v>0.0636679083108902</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.06671114265918732</c:v>
+                  <c:v>0.0636679083108902</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.06004002690315247</c:v>
+                  <c:v>0.0573011189699173</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.06004002690315247</c:v>
+                  <c:v>0.0573011189699173</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.06004002690315247</c:v>
+                  <c:v>0.0573011189699173</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.06004002690315247</c:v>
+                  <c:v>0.0573011189699173</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.05336891114711762</c:v>
+                  <c:v>0.0509343259036541</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.05336891114711762</c:v>
+                  <c:v>0.0509343259036541</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.05003335699439049</c:v>
+                  <c:v>0.04775093123316765</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.05003335699439049</c:v>
+                  <c:v>0.04775093123316765</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.05003335699439049</c:v>
+                  <c:v>0.04775093123316765</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.04669779911637306</c:v>
+                  <c:v>0.0445675365626812</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.04669779911637306</c:v>
+                  <c:v>0.0445675365626812</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0.04336224123835564</c:v>
+                  <c:v>0.04138414189219475</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0.04002668336033821</c:v>
+                  <c:v>0.04138414189219475</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>0.04002668336033821</c:v>
+                  <c:v>0.038200743496418</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>0.03335557132959366</c:v>
+                  <c:v>0.038200743496418</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>0.03002001345157623</c:v>
+                  <c:v>0.0318339541554451</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>0.02334889955818653</c:v>
+                  <c:v>0.02865055948495865</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>0.02001334168016911</c:v>
+                  <c:v>0.0222837682813406</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>0.0133422277867794</c:v>
+                  <c:v>0.019100371748209</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>0.0133422277867794</c:v>
+                  <c:v>0.01273358147591353</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>0.006671113893389702</c:v>
+                  <c:v>0.01273358147591353</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>0.006671113893389702</c:v>
+                  <c:v>0.006366790737956762</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>0.006671113893389702</c:v>
+                  <c:v>0.006366790737956762</c:v>
                 </c:pt>
                 <c:pt idx="53">
+                  <c:v>0.006366790737956762</c:v>
+                </c:pt>
+                <c:pt idx="54">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -853,8 +862,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H56" totalsRowCount="1">
-  <autoFilter ref="A2:H55"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H57" totalsRowCount="1">
+  <autoFilter ref="A2:H56"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="ram_percent" totalsRowFunction="sum"/>
@@ -870,8 +879,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H56" totalsRowCount="1">
-  <autoFilter ref="A2:H55"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H57" totalsRowCount="1">
+  <autoFilter ref="A2:H56"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="flash_percent" totalsRowFunction="sum"/>
@@ -1171,7 +1180,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1184,28 +1193,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1213,25 +1222,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>97.79456329345703</v>
+        <v>97.96974182128906</v>
       </c>
       <c r="C3" s="1">
-        <v>46471</v>
+        <v>50571</v>
       </c>
       <c r="D3" s="1">
-        <v>44282</v>
+        <v>47096</v>
       </c>
       <c r="E3" s="1">
-        <v>40688</v>
+        <v>43200</v>
       </c>
       <c r="F3" s="1">
-        <v>3395</v>
+        <v>3697</v>
       </c>
       <c r="G3" s="1">
         <v>199</v>
       </c>
       <c r="H3" s="1">
-        <v>46272</v>
+        <v>50372</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1239,7 +1248,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>2.154927492141724</v>
+        <v>1.983765721321106</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1265,16 +1274,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="2">
-        <v>0.0252530574798584</v>
+        <v>0.02324725314974785</v>
       </c>
       <c r="C5" s="1">
         <v>12</v>
       </c>
       <c r="D5" s="1">
-        <v>6355</v>
+        <v>6381</v>
       </c>
       <c r="E5" s="1">
-        <v>6210</v>
+        <v>6236</v>
       </c>
       <c r="F5" s="1">
         <v>133</v>
@@ -1291,7 +1300,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.008417685516178608</v>
+        <v>0.00774908484891057</v>
       </c>
       <c r="C6" s="1">
         <v>4</v>
@@ -1317,7 +1326,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.008417685516178608</v>
+        <v>0.00774908484891057</v>
       </c>
       <c r="C7" s="1">
         <v>4</v>
@@ -1343,7 +1352,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.008417685516178608</v>
+        <v>0.00774908484891057</v>
       </c>
       <c r="C8" s="1">
         <v>4</v>
@@ -1364,35 +1373,35 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
-      <c r="A56" t="s">
-        <v>55</v>
-      </c>
-      <c r="B56">
+    <row r="57" spans="1:8">
+      <c r="A57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B57">
         <f>SUBTOTAL(109,[ram_percent])</f>
         <v>0</v>
       </c>
-      <c r="C56">
+      <c r="C57">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="D56">
+      <c r="D57">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="E56">
+      <c r="E57">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F56">
+      <c r="F57">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G56">
+      <c r="G57">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H56">
+      <c r="H57">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>
@@ -1408,7 +1417,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1421,28 +1430,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" t="s">
         <v>63</v>
-      </c>
-      <c r="C2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1450,25 +1459,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>73.85256958007813</v>
+        <v>74.96259307861328</v>
       </c>
       <c r="C3" s="1">
-        <v>44282</v>
+        <v>47096</v>
       </c>
       <c r="D3" s="1">
-        <v>46471</v>
+        <v>50571</v>
       </c>
       <c r="E3" s="1">
-        <v>40688</v>
+        <v>43200</v>
       </c>
       <c r="F3" s="1">
-        <v>3395</v>
+        <v>3697</v>
       </c>
       <c r="G3" s="1">
         <v>199</v>
       </c>
       <c r="H3" s="1">
-        <v>46272</v>
+        <v>50372</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1476,16 +1485,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>10.59873294830322</v>
+        <v>10.15662288665772</v>
       </c>
       <c r="C4" s="1">
-        <v>6355</v>
+        <v>6381</v>
       </c>
       <c r="D4" s="1">
         <v>12</v>
       </c>
       <c r="E4" s="1">
-        <v>6210</v>
+        <v>6236</v>
       </c>
       <c r="F4" s="1">
         <v>133</v>
@@ -1502,7 +1511,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="2">
-        <v>3.889259576797485</v>
+        <v>3.711838960647583</v>
       </c>
       <c r="C5" s="1">
         <v>2332</v>
@@ -1528,7 +1537,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="2">
-        <v>2.094729900360107</v>
+        <v>1.999172329902649</v>
       </c>
       <c r="C6" s="1">
         <v>1256</v>
@@ -1554,7 +1563,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="2">
-        <v>1.464309573173523</v>
+        <v>1.397510528564453</v>
       </c>
       <c r="C7" s="1">
         <v>878</v>
@@ -1580,7 +1589,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="2">
-        <v>1.354236125946045</v>
+        <v>1.292458534240723</v>
       </c>
       <c r="C8" s="1">
         <v>812</v>
@@ -1606,7 +1615,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="2">
-        <v>0.7071381211280823</v>
+        <v>0.6748798489570618</v>
       </c>
       <c r="C9" s="1">
         <v>424</v>
@@ -1632,7 +1641,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="2">
-        <v>0.5703802704811096</v>
+        <v>0.5443606376647949</v>
       </c>
       <c r="C10" s="1">
         <v>342</v>
@@ -1658,7 +1667,7 @@
         <v>12</v>
       </c>
       <c r="B11" s="2">
-        <v>0.5570380091667175</v>
+        <v>0.5316270589828491</v>
       </c>
       <c r="C11" s="1">
         <v>334</v>
@@ -1684,7 +1693,7 @@
         <v>13</v>
       </c>
       <c r="B12" s="2">
-        <v>0.5537024736404419</v>
+        <v>0.5284436345100403</v>
       </c>
       <c r="C12" s="1">
         <v>332</v>
@@ -1710,7 +1719,7 @@
         <v>14</v>
       </c>
       <c r="B13" s="2">
-        <v>0.3802534937858582</v>
+        <v>0.3629070818424225</v>
       </c>
       <c r="C13" s="1">
         <v>228</v>
@@ -1736,7 +1745,7 @@
         <v>15</v>
       </c>
       <c r="B14" s="2">
-        <v>0.3735823929309845</v>
+        <v>0.3565402925014496</v>
       </c>
       <c r="C14" s="1">
         <v>224</v>
@@ -1762,7 +1771,7 @@
         <v>16</v>
       </c>
       <c r="B15" s="2">
-        <v>0.3702468276023865</v>
+        <v>0.3533568978309631</v>
       </c>
       <c r="C15" s="1">
         <v>222</v>
@@ -1788,7 +1797,7 @@
         <v>17</v>
       </c>
       <c r="B16" s="2">
-        <v>0.310206800699234</v>
+        <v>0.2960557639598846</v>
       </c>
       <c r="C16" s="1">
         <v>186</v>
@@ -1814,7 +1823,7 @@
         <v>18</v>
       </c>
       <c r="B17" s="2">
-        <v>0.2635090053081513</v>
+        <v>0.2514882385730743</v>
       </c>
       <c r="C17" s="1">
         <v>158</v>
@@ -1840,7 +1849,7 @@
         <v>19</v>
       </c>
       <c r="B18" s="2">
-        <v>0.235156774520874</v>
+        <v>0.2244293689727783</v>
       </c>
       <c r="C18" s="1">
         <v>141</v>
@@ -1866,7 +1875,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="2">
-        <v>0.1867911964654923</v>
+        <v>0.1782701462507248</v>
       </c>
       <c r="C19" s="1">
         <v>112</v>
@@ -1892,7 +1901,7 @@
         <v>21</v>
       </c>
       <c r="B20" s="2">
-        <v>0.1834556311368942</v>
+        <v>0.1750867515802383</v>
       </c>
       <c r="C20" s="1">
         <v>110</v>
@@ -1918,7 +1927,7 @@
         <v>22</v>
       </c>
       <c r="B21" s="2">
-        <v>0.1634422987699509</v>
+        <v>0.1559863686561585</v>
       </c>
       <c r="C21" s="1">
         <v>98</v>
@@ -1944,7 +1953,7 @@
         <v>23</v>
       </c>
       <c r="B22" s="2">
-        <v>0.1634422987699509</v>
+        <v>0.1559863686561585</v>
       </c>
       <c r="C22" s="1">
         <v>98</v>
@@ -1970,7 +1979,7 @@
         <v>4</v>
       </c>
       <c r="B23" s="2">
-        <v>0.1200800538063049</v>
+        <v>0.1146022379398346</v>
       </c>
       <c r="C23" s="1">
         <v>72</v>
@@ -1996,7 +2005,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="2">
-        <v>0.1067378222942352</v>
+        <v>0.1018686518073082</v>
       </c>
       <c r="C24" s="1">
         <v>64</v>
@@ -2022,7 +2031,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="2">
-        <v>0.09339559823274612</v>
+        <v>0.0891350731253624</v>
       </c>
       <c r="C25" s="1">
         <v>56</v>
@@ -2048,7 +2057,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="2">
-        <v>0.09339559823274612</v>
+        <v>0.0891350731253624</v>
       </c>
       <c r="C26" s="1">
         <v>56</v>
@@ -2074,7 +2083,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="2">
-        <v>0.08005336672067642</v>
+        <v>0.076401486992836</v>
       </c>
       <c r="C27" s="1">
         <v>48</v>
@@ -2100,7 +2109,7 @@
         <v>28</v>
       </c>
       <c r="B28" s="2">
-        <v>0.08005336672067642</v>
+        <v>0.076401486992836</v>
       </c>
       <c r="C28" s="1">
         <v>48</v>
@@ -2126,7 +2135,7 @@
         <v>29</v>
       </c>
       <c r="B29" s="2">
-        <v>0.08005336672067642</v>
+        <v>0.076401486992836</v>
       </c>
       <c r="C29" s="1">
         <v>48</v>
@@ -2152,7 +2161,7 @@
         <v>30</v>
       </c>
       <c r="B30" s="2">
-        <v>0.07338225841522217</v>
+        <v>0.0700346976518631</v>
       </c>
       <c r="C30" s="1">
         <v>44</v>
@@ -2178,7 +2187,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="2">
-        <v>0.06671114265918732</v>
+        <v>0.0636679083108902</v>
       </c>
       <c r="C31" s="1">
         <v>40</v>
@@ -2204,7 +2213,7 @@
         <v>32</v>
       </c>
       <c r="B32" s="2">
-        <v>0.06671114265918732</v>
+        <v>0.0636679083108902</v>
       </c>
       <c r="C32" s="1">
         <v>40</v>
@@ -2230,7 +2239,7 @@
         <v>33</v>
       </c>
       <c r="B33" s="2">
-        <v>0.06004002690315247</v>
+        <v>0.0573011189699173</v>
       </c>
       <c r="C33" s="1">
         <v>36</v>
@@ -2256,7 +2265,7 @@
         <v>34</v>
       </c>
       <c r="B34" s="2">
-        <v>0.06004002690315247</v>
+        <v>0.0573011189699173</v>
       </c>
       <c r="C34" s="1">
         <v>36</v>
@@ -2282,7 +2291,7 @@
         <v>35</v>
       </c>
       <c r="B35" s="2">
-        <v>0.06004002690315247</v>
+        <v>0.0573011189699173</v>
       </c>
       <c r="C35" s="1">
         <v>36</v>
@@ -2308,7 +2317,7 @@
         <v>36</v>
       </c>
       <c r="B36" s="2">
-        <v>0.06004002690315247</v>
+        <v>0.0573011189699173</v>
       </c>
       <c r="C36" s="1">
         <v>36</v>
@@ -2334,7 +2343,7 @@
         <v>37</v>
       </c>
       <c r="B37" s="2">
-        <v>0.05336891114711762</v>
+        <v>0.0509343259036541</v>
       </c>
       <c r="C37" s="1">
         <v>32</v>
@@ -2360,7 +2369,7 @@
         <v>38</v>
       </c>
       <c r="B38" s="2">
-        <v>0.05336891114711762</v>
+        <v>0.0509343259036541</v>
       </c>
       <c r="C38" s="1">
         <v>32</v>
@@ -2386,7 +2395,7 @@
         <v>39</v>
       </c>
       <c r="B39" s="2">
-        <v>0.05003335699439049</v>
+        <v>0.04775093123316765</v>
       </c>
       <c r="C39" s="1">
         <v>30</v>
@@ -2412,7 +2421,7 @@
         <v>40</v>
       </c>
       <c r="B40" s="2">
-        <v>0.05003335699439049</v>
+        <v>0.04775093123316765</v>
       </c>
       <c r="C40" s="1">
         <v>30</v>
@@ -2438,7 +2447,7 @@
         <v>41</v>
       </c>
       <c r="B41" s="2">
-        <v>0.05003335699439049</v>
+        <v>0.04775093123316765</v>
       </c>
       <c r="C41" s="1">
         <v>30</v>
@@ -2464,7 +2473,7 @@
         <v>42</v>
       </c>
       <c r="B42" s="2">
-        <v>0.04669779911637306</v>
+        <v>0.0445675365626812</v>
       </c>
       <c r="C42" s="1">
         <v>28</v>
@@ -2490,7 +2499,7 @@
         <v>43</v>
       </c>
       <c r="B43" s="2">
-        <v>0.04669779911637306</v>
+        <v>0.0445675365626812</v>
       </c>
       <c r="C43" s="1">
         <v>28</v>
@@ -2516,7 +2525,7 @@
         <v>44</v>
       </c>
       <c r="B44" s="2">
-        <v>0.04336224123835564</v>
+        <v>0.04138414189219475</v>
       </c>
       <c r="C44" s="1">
         <v>26</v>
@@ -2542,16 +2551,16 @@
         <v>45</v>
       </c>
       <c r="B45" s="2">
-        <v>0.04002668336033821</v>
+        <v>0.04138414189219475</v>
       </c>
       <c r="C45" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D45" s="1">
         <v>0</v>
       </c>
       <c r="E45" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F45" s="1">
         <v>0</v>
@@ -2568,7 +2577,7 @@
         <v>46</v>
       </c>
       <c r="B46" s="2">
-        <v>0.04002668336033821</v>
+        <v>0.038200743496418</v>
       </c>
       <c r="C46" s="1">
         <v>24</v>
@@ -2594,16 +2603,16 @@
         <v>47</v>
       </c>
       <c r="B47" s="2">
-        <v>0.03335557132959366</v>
+        <v>0.038200743496418</v>
       </c>
       <c r="C47" s="1">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D47" s="1">
         <v>0</v>
       </c>
       <c r="E47" s="1">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F47" s="1">
         <v>0</v>
@@ -2620,16 +2629,16 @@
         <v>48</v>
       </c>
       <c r="B48" s="2">
-        <v>0.03002001345157623</v>
+        <v>0.0318339541554451</v>
       </c>
       <c r="C48" s="1">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D48" s="1">
         <v>0</v>
       </c>
       <c r="E48" s="1">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F48" s="1">
         <v>0</v>
@@ -2646,16 +2655,16 @@
         <v>49</v>
       </c>
       <c r="B49" s="2">
-        <v>0.02334889955818653</v>
+        <v>0.02865055948495865</v>
       </c>
       <c r="C49" s="1">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D49" s="1">
         <v>0</v>
       </c>
       <c r="E49" s="1">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F49" s="1">
         <v>0</v>
@@ -2669,25 +2678,25 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="1" t="s">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="B50" s="2">
-        <v>0.02001334168016911</v>
+        <v>0.0222837682813406</v>
       </c>
       <c r="C50" s="1">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D50" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E50" s="1">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F50" s="1">
         <v>0</v>
       </c>
       <c r="G50" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H50" s="1">
         <v>0</v>
@@ -2695,16 +2704,16 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="1" t="s">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="B51" s="2">
-        <v>0.0133422277867794</v>
+        <v>0.019100371748209</v>
       </c>
       <c r="C51" s="1">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D51" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E51" s="1">
         <v>8</v>
@@ -2713,7 +2722,7 @@
         <v>0</v>
       </c>
       <c r="G51" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H51" s="1">
         <v>0</v>
@@ -2724,7 +2733,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="2">
-        <v>0.0133422277867794</v>
+        <v>0.01273358147591353</v>
       </c>
       <c r="C52" s="1">
         <v>8</v>
@@ -2747,25 +2756,25 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="1" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="B53" s="2">
-        <v>0.006671113893389702</v>
+        <v>0.01273358147591353</v>
       </c>
       <c r="C53" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D53" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E53" s="1">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F53" s="1">
         <v>0</v>
       </c>
       <c r="G53" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H53" s="1">
         <v>0</v>
@@ -2773,25 +2782,25 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="1" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="B54" s="2">
-        <v>0.006671113893389702</v>
+        <v>0.006366790737956762</v>
       </c>
       <c r="C54" s="1">
         <v>4</v>
       </c>
       <c r="D54" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E54" s="1">
+        <v>0</v>
+      </c>
+      <c r="F54" s="1">
+        <v>0</v>
+      </c>
+      <c r="G54" s="1">
         <v>4</v>
-      </c>
-      <c r="F54" s="1">
-        <v>0</v>
-      </c>
-      <c r="G54" s="1">
-        <v>0</v>
       </c>
       <c r="H54" s="1">
         <v>0</v>
@@ -2802,7 +2811,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="2">
-        <v>0.006671113893389702</v>
+        <v>0.006366790737956762</v>
       </c>
       <c r="C55" s="1">
         <v>4</v>
@@ -2824,34 +2833,60 @@
       </c>
     </row>
     <row r="56" spans="1:8">
-      <c r="A56" t="s">
-        <v>55</v>
-      </c>
-      <c r="B56">
+      <c r="A56" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" s="2">
+        <v>0.006366790737956762</v>
+      </c>
+      <c r="C56" s="1">
+        <v>4</v>
+      </c>
+      <c r="D56" s="1">
+        <v>0</v>
+      </c>
+      <c r="E56" s="1">
+        <v>4</v>
+      </c>
+      <c r="F56" s="1">
+        <v>0</v>
+      </c>
+      <c r="G56" s="1">
+        <v>0</v>
+      </c>
+      <c r="H56" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B57">
         <f>SUBTOTAL(109,[flash_percent])</f>
         <v>0</v>
       </c>
-      <c r="C56">
+      <c r="C57">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="D56">
+      <c r="D57">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="E56">
+      <c r="E57">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F56">
+      <c r="F57">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G56">
+      <c r="G57">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H56">
+      <c r="H57">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>

</xml_diff>